<commit_message>
v2.1: Sync E drive canonical repo
</commit_message>
<xml_diff>
--- a/04_图表/Table_TB_Divergence_Statistics.xlsx
+++ b/04_图表/Table_TB_Divergence_Statistics.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +37,10 @@
     <font>
       <name val="Arial"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="FF999999"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="4">
@@ -59,7 +63,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -81,11 +85,17 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -96,6 +106,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -461,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -778,6 +789,13 @@
       </c>
       <c r="L7" s="3" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>（内容由AI生成，仅供参考）</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>